<commit_message>
Align guide and tracker with revised agenda times (9:00-4:00 days, 12-1 lunch)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01W6mJ1brKLV5iN37yui29cR
</commit_message>
<xml_diff>
--- a/ezurio-onsite-prep/03_Ezurio_Requirements_and_Observations_Tracker.xlsx
+++ b/ezurio-onsite-prep/03_Ezurio_Requirements_and_Observations_Tracker.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'2 Observations'!$A$1:$K$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'3 Irvine Backlog'!$A$1:$J$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'4 GWTrack Features'!$A$1:$K$25</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'6 Open Items'!$A$1:$E$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'6 Open Items'!$A$1:$E$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -3831,7 +3831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -4087,32 +4087,59 @@
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
+          <t>OI-010</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Agenda fix: Day 2 session 2.3 still starts 12:45 but lunch now runs 12:00–1:00 – confirm 2.3 = 1:00–2:45</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Jordan Piatek</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>Before sending agenda</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
           <t>OI-009</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>Confirm why Auto-Mark WOs Built workflow was suspended 10/1 and current WO closing process</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>Trevor Kanwal / Ezurio</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
+      <c r="D11" s="4" t="inlineStr">
         <is>
           <t>Before 10/21</t>
         </is>
       </c>
-      <c r="E10" s="4" t="inlineStr">
+      <c r="E11" s="4" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E10"/>
+  <autoFilter ref="A1:E11"/>
   <dataValidations count="1">
     <dataValidation sqref="E2:E300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Open,In progress,Done,Blocked"</formula1>

</xml_diff>